<commit_message>
Google vs bodhi gateway
</commit_message>
<xml_diff>
--- a/output/intraday_tracker.xlsx
+++ b/output/intraday_tracker.xlsx
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -514,6 +514,11 @@
           <t>2026-09-03</t>
         </is>
       </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -570,6 +575,11 @@
           <t>₹11,920.00 (-0.7%)</t>
         </is>
       </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>₹11,800.00 (-1.0%)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -626,6 +636,11 @@
           <t>₹1,319.00 (-0.9%)</t>
         </is>
       </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>₹1,282.80 (-2.7%)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -682,6 +697,11 @@
           <t>₹3,150.00 (-0.9%)</t>
         </is>
       </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>₹3,160.00 (+0.3%)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -736,6 +756,11 @@
       <c r="L6" t="inlineStr">
         <is>
           <t>₹1,302.50 (-0.4%)</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>₹1,309.50 (+0.5%)</t>
         </is>
       </c>
     </row>

</xml_diff>